<commit_message>
Fixed upload excel functions
</commit_message>
<xml_diff>
--- a/template/Supplier_Template.xlsx
+++ b/template/Supplier_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jihbi\xampp\htdocs\synctronix\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/syncweigh-wb/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6F1D70-470F-440C-8113-583ADE3EBD6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{420B215E-6467-784F-9286-D65D92CAD93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{5422817E-FF8F-45E7-AD6A-87189E46CF41}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" xr2:uid="{5422817E-FF8F-45E7-AD6A-87189E46CF41}"/>
   </bookViews>
   <sheets>
     <sheet name="bl_vendor" sheetId="1" r:id="rId1"/>
@@ -408,23 +408,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51F75F9-0BCD-457C-BDCB-0EB3FC71AA51}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="60.42578125" customWidth="1"/>
-    <col min="8" max="8" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>

</xml_diff>